<commit_message>
test: add E2E tests, TestingPlan, BugReport; update frontend UI
</commit_message>
<xml_diff>
--- a/test/NCKH_TestCase.xlsx
+++ b/test/NCKH_TestCase.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9060" activeTab="3"/>
+    <workbookView windowWidth="23040" windowHeight="8400"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="620" uniqueCount="388">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="651" uniqueCount="405">
   <si>
     <t>TEST CASE — AI LEGAL INTELLIGENCE PLATFORM</t>
   </si>
@@ -55,7 +55,7 @@
     <t>Tên dự án:</t>
   </si>
   <si>
-    <t>AI Legal Intelligence Platform — Tìm kiếm &amp; Hỏi đáp Pháp luật Việt Nam</t>
+    <t>AI Legal Intelligence Platform - Nền tảng Tìm kiếm &amp; Hỏi đáp Pháp luật Việt Nam</t>
   </si>
   <si>
     <t>Nguồn dữ liệu:</t>
@@ -100,9 +100,6 @@
     <t>Khởi tạo file Test Case, bao gồm 7 module: AUTH, SEARCH, AI-RAG, DOC, WORKSPACE, ANALYTICS, NON-FUNC</t>
   </si>
   <si>
-    <t>Nhóm NCKH</t>
-  </si>
-  <si>
     <t>GVHD</t>
   </si>
   <si>
@@ -127,19 +124,19 @@
     <t>Phụ trách module</t>
   </si>
   <si>
-    <t>[Họ tên thành viên 1]</t>
+    <t>Vũ Lưu Minh Toàn</t>
+  </si>
+  <si>
+    <t>Trưởng nhóm / Dev</t>
+  </si>
+  <si>
+    <t>AUTH, SEARCH, AI-RAG</t>
+  </si>
+  <si>
+    <t>[Họ tên thành viên 2]</t>
   </si>
   <si>
     <t>[MSSV]</t>
-  </si>
-  <si>
-    <t>Trưởng nhóm / Dev</t>
-  </si>
-  <si>
-    <t>AUTH, SEARCH, AI-RAG</t>
-  </si>
-  <si>
-    <t>[Họ tên thành viên 2]</t>
   </si>
   <si>
     <t>Dev / Tester</t>
@@ -699,6 +696,26 @@
     <t>Keyboard shortcut UX</t>
   </si>
   <si>
+    <t>Validation khi để trống ô tìm kiếm</t>
+  </si>
+  <si>
+    <t>Không có điều kiện đặc biệt</t>
+  </si>
+  <si>
+    <t>1. Vào trang Tìm kiếm
+2. Để trống ô tìm kiếm
+3. Click Tìm kiếm</t>
+  </si>
+  <si>
+    <t>[Empty]</t>
+  </si>
+  <si>
+    <t>Nút tìm kiếm bị disable hoặc xuất hiện cảnh báo. Không gọi API.</t>
+  </si>
+  <si>
+    <t>Negative Test - UI Validation</t>
+  </si>
+  <si>
     <t>MODULE: MODULE 3: AI CHAT &amp; RAG ENGINE</t>
   </si>
   <si>
@@ -868,6 +885,27 @@
     <t>API: POST /ai/summarize</t>
   </si>
   <si>
+    <t>AI Chat - Security</t>
+  </si>
+  <si>
+    <t>Rate Limiting (Chống Spam)</t>
+  </si>
+  <si>
+    <t>Đã đăng nhập</t>
+  </si>
+  <si>
+    <t>1. Cố tình click nút Gửi tin nhắn liên tục 10 lần/giây</t>
+  </si>
+  <si>
+    <t>Spam click liên tục</t>
+  </si>
+  <si>
+    <t>API chặn lại, trả về mã lỗi HTTP 429 Too Many Requests. Frontend hiện cảnh báo.</t>
+  </si>
+  <si>
+    <t>DDoS Prevention</t>
+  </si>
+  <si>
     <t>MODULE: MODULE 4: XEM CHI TIẾT VĂN BẢN &amp; KNOWLEDGE GRAPH</t>
   </si>
   <si>
@@ -955,9 +993,6 @@
   </si>
   <si>
     <t>Mở văn bản bằng ID không tồn tại</t>
-  </si>
-  <si>
-    <t>Đã đăng nhập</t>
   </si>
   <si>
     <t>1. Truy cập trực tiếp URL: http://localhost:5173/documents/99999999</t>
@@ -1362,6 +1397,26 @@
   </si>
   <si>
     <t>JWT exp claim validation</t>
+  </si>
+  <si>
+    <t>Bảo mật — XSS</t>
+  </si>
+  <si>
+    <t>Hệ thống miễn nhiễm với XSS Injection trên form Search</t>
+  </si>
+  <si>
+    <t>1. Vào ô tìm kiếm
+2. Nhập mã độc XSS
+3. Bấm tìm kiếm</t>
+  </si>
+  <si>
+    <t>keyword: &lt;script&gt;alert('Hacked')&lt;/script&gt;</t>
+  </si>
+  <si>
+    <t>Mã độc bị Frontend tự động encode. Không hiển thị popup alert.</t>
+  </si>
+  <si>
+    <t>XSS Prevention</t>
   </si>
 </sst>
 </file>
@@ -1374,7 +1429,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="40">
+  <fonts count="39">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1510,13 +1565,6 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <u/>
@@ -1893,7 +1941,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -1905,6 +1953,19 @@
       <left style="thin">
         <color rgb="FFCCCCCC"/>
       </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right style="thin">
         <color rgb="FFCCCCCC"/>
       </right>
@@ -2017,152 +2078,152 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="20" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="20" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="20" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="20" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="20" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="8" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="3">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="4">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="4">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="5">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="9" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="9" borderId="6">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="10" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="10" borderId="7">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="10" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="10" borderId="6">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="11" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="11" borderId="8">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="9">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="10">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="34" fillId="12" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="35" fillId="13" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="36" fillId="14" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="37" fillId="15" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="38" fillId="16" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="38" fillId="17" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="37" fillId="18" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="37" fillId="19" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="38" fillId="20" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="38" fillId="21" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="37" fillId="22" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="37" fillId="23" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="38" fillId="24" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="38" fillId="25" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="37" fillId="26" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="37" fillId="27" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="38" fillId="28" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="38" fillId="29" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="37" fillId="30" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="37" fillId="31" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="38" fillId="32" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="38" fillId="33" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="37" fillId="34" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="37" fillId="35" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="38" fillId="36" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="38" fillId="37" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="37" fillId="38" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2231,6 +2292,7 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2336,6 +2398,9 @@
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -2377,6 +2442,7 @@
         <a:noFill/>
         <a:ln w="9525">
           <a:noFill/>
+          <a:prstDash val="solid"/>
         </a:ln>
       </xdr:spPr>
     </xdr:pic>
@@ -2419,6 +2485,7 @@
         <a:noFill/>
         <a:ln w="9525">
           <a:noFill/>
+          <a:prstDash val="solid"/>
         </a:ln>
       </xdr:spPr>
     </xdr:pic>
@@ -2461,6 +2528,7 @@
         <a:noFill/>
         <a:ln w="9525">
           <a:noFill/>
+          <a:prstDash val="solid"/>
         </a:ln>
       </xdr:spPr>
     </xdr:pic>
@@ -2503,6 +2571,7 @@
         <a:noFill/>
         <a:ln w="9525">
           <a:noFill/>
+          <a:prstDash val="solid"/>
         </a:ln>
       </xdr:spPr>
     </xdr:pic>
@@ -2545,6 +2614,7 @@
         <a:noFill/>
         <a:ln w="9525">
           <a:noFill/>
+          <a:prstDash val="solid"/>
         </a:ln>
       </xdr:spPr>
     </xdr:pic>
@@ -2587,6 +2657,7 @@
         <a:noFill/>
         <a:ln w="9525">
           <a:noFill/>
+          <a:prstDash val="solid"/>
         </a:ln>
       </xdr:spPr>
     </xdr:pic>
@@ -2629,6 +2700,7 @@
         <a:noFill/>
         <a:ln w="9525">
           <a:noFill/>
+          <a:prstDash val="solid"/>
         </a:ln>
       </xdr:spPr>
     </xdr:pic>
@@ -2935,7 +3007,7 @@
   </cols>
   <sheetData>
     <row r="2" ht="36" customHeight="1" spans="2:8">
-      <c r="B2" s="26" t="s">
+      <c r="B2" s="27" t="s">
         <v>0</v>
       </c>
     </row>
@@ -2943,7 +3015,7 @@
       <c r="B3" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="27" t="s">
+      <c r="D3" s="28" t="s">
         <v>2</v>
       </c>
     </row>
@@ -2951,7 +3023,7 @@
       <c r="B4" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="28" t="s">
+      <c r="D4" s="29" t="s">
         <v>4</v>
       </c>
     </row>
@@ -2967,7 +3039,7 @@
       <c r="B6" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="D6" s="28" t="s">
+      <c r="D6" s="29" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2975,7 +3047,7 @@
       <c r="B7" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="D7" s="28" t="s">
+      <c r="D7" s="29" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2986,25 +3058,25 @@
       </c>
     </row>
     <row r="10" ht="20" customHeight="1" spans="2:8">
-      <c r="B10" s="29" t="s">
+      <c r="B10" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="29" t="s">
+      <c r="C10" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="D10" s="29" t="s">
+      <c r="D10" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="E10" s="29" t="s">
+      <c r="E10" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="29" t="s">
+      <c r="F10" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="G10" s="29" t="s">
+      <c r="G10" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="H10" s="29" t="s">
+      <c r="H10" s="30" t="s">
         <v>18</v>
       </c>
     </row>
@@ -3021,37 +3093,35 @@
       <c r="E11" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="F11" s="18" t="s">
+      <c r="F11" s="18"/>
+      <c r="G11" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="G11" s="18" t="s">
+      <c r="H11" s="18" t="s">
         <v>22</v>
-      </c>
-      <c r="H11" s="18" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="13" ht="16" customHeight="1"/>
     <row r="14" ht="24" customHeight="1" spans="2:8">
       <c r="B14" s="23" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1" spans="2:8">
+      <c r="B15" s="30" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="15" ht="20" customHeight="1" spans="2:8">
-      <c r="B15" s="29" t="s">
+      <c r="C15" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="29" t="s">
+      <c r="D15" s="30" t="s">
         <v>26</v>
       </c>
-      <c r="D15" s="29" t="s">
+      <c r="E15" s="30" t="s">
         <v>27</v>
       </c>
-      <c r="E15" s="29" t="s">
+      <c r="F15" s="30" t="s">
         <v>28</v>
-      </c>
-      <c r="F15" s="29" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1" spans="2:8">
@@ -3059,16 +3129,16 @@
         <v>1</v>
       </c>
       <c r="C16" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="D16" s="18">
+        <v>2354050139</v>
+      </c>
+      <c r="E16" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="D16" s="18" t="s">
+      <c r="F16" s="18" t="s">
         <v>31</v>
-      </c>
-      <c r="E16" s="18" t="s">
-        <v>32</v>
-      </c>
-      <c r="F16" s="18" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1" spans="2:6">
@@ -3076,16 +3146,16 @@
         <v>2</v>
       </c>
       <c r="C17" s="21" t="s">
+        <v>32</v>
+      </c>
+      <c r="D17" s="21" t="s">
+        <v>33</v>
+      </c>
+      <c r="E17" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="D17" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="E17" s="21" t="s">
+      <c r="F17" s="21" t="s">
         <v>35</v>
-      </c>
-      <c r="F17" s="21" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1" spans="2:6">
@@ -3093,16 +3163,16 @@
         <v>3</v>
       </c>
       <c r="C18" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="D18" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="E18" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="F18" s="18" t="s">
         <v>37</v>
-      </c>
-      <c r="D18" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="E18" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="F18" s="18" t="s">
-        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -3131,7 +3201,7 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
-    <col min="2" max="2" width="5" customWidth="1"/>
+    <col min="2" max="2" width="15.6666666666667" customWidth="1"/>
     <col min="3" max="3" width="30" customWidth="1"/>
     <col min="4" max="8" width="14" customWidth="1"/>
     <col min="9" max="9" width="18" customWidth="1"/>
@@ -3139,20 +3209,20 @@
   <sheetData>
     <row r="2" ht="34" customHeight="1" spans="2:9">
       <c r="B2" s="11" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="2:9">
       <c r="B3" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="C3" s="13" t="s">
         <v>40</v>
-      </c>
-      <c r="C3" s="13" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="4" spans="2:9">
       <c r="B4" s="14" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C4" s="15" t="s">
         <v>4</v>
@@ -3167,25 +3237,25 @@
     <row r="5" ht="14" customHeight="1"/>
     <row r="6" ht="22" customHeight="1" spans="2:9">
       <c r="B6" s="16" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C6" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="D6" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="D6" s="16" t="s">
+      <c r="E6" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="E6" s="16" t="s">
+      <c r="F6" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="F6" s="16" t="s">
+      <c r="G6" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="G6" s="16" t="s">
+      <c r="H6" s="16" t="s">
         <v>47</v>
-      </c>
-      <c r="H6" s="16" t="s">
-        <v>48</v>
       </c>
       <c r="I6" s="16" t="s">
         <v>18</v>
@@ -3196,7 +3266,7 @@
         <v>1</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D7" s="17">
         <v>6</v>
@@ -3211,10 +3281,10 @@
         <v>0</v>
       </c>
       <c r="H7" s="17" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I7" s="17" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1" spans="2:9">
@@ -3222,7 +3292,7 @@
         <v>2</v>
       </c>
       <c r="C8" s="21" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D8" s="20">
         <v>6</v>
@@ -3237,10 +3307,10 @@
         <v>0</v>
       </c>
       <c r="H8" s="20" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I8" s="20" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1" spans="2:9">
@@ -3248,7 +3318,7 @@
         <v>3</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D9" s="17">
         <v>6</v>
@@ -3263,10 +3333,10 @@
         <v>0</v>
       </c>
       <c r="H9" s="17" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I9" s="17" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1" spans="2:9">
@@ -3274,7 +3344,7 @@
         <v>4</v>
       </c>
       <c r="C10" s="21" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D10" s="20">
         <v>3</v>
@@ -3289,10 +3359,10 @@
         <v>0</v>
       </c>
       <c r="H10" s="20" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I10" s="20" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1" spans="2:9">
@@ -3300,7 +3370,7 @@
         <v>5</v>
       </c>
       <c r="C11" s="18" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D11" s="17">
         <v>6</v>
@@ -3315,10 +3385,10 @@
         <v>0</v>
       </c>
       <c r="H11" s="17" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I11" s="17" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1" spans="2:9">
@@ -3326,7 +3396,7 @@
         <v>6</v>
       </c>
       <c r="C12" s="21" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D12" s="20">
         <v>2</v>
@@ -3341,10 +3411,10 @@
         <v>0</v>
       </c>
       <c r="H12" s="20" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I12" s="20" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1" spans="2:9">
@@ -3352,7 +3422,7 @@
         <v>7</v>
       </c>
       <c r="C13" s="18" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D13" s="17">
         <v>5</v>
@@ -3367,18 +3437,18 @@
         <v>0</v>
       </c>
       <c r="H13" s="17" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I13" s="17" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1" spans="2:9">
       <c r="B14" s="16" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C14" s="22" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D14" s="16">
         <v>34</v>
@@ -3393,64 +3463,70 @@
         <v>0</v>
       </c>
       <c r="H14" s="16" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I14" s="16" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1" spans="2:9">
       <c r="B16" s="23" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="17" ht="39" customHeight="1" spans="2:4">
+      <c r="B17" s="24" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="17" ht="18" customHeight="1" spans="2:3">
-      <c r="B17" s="24" t="s">
+      <c r="C17" s="25" t="s">
         <v>59</v>
       </c>
-      <c r="C17" s="25" t="s">
+      <c r="D17" s="26"/>
+    </row>
+    <row r="18" ht="18" customHeight="1" spans="2:4">
+      <c r="B18" s="24" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="18" ht="18" customHeight="1" spans="2:3">
-      <c r="B18" s="24" t="s">
+      <c r="C18" s="25" t="s">
+        <v>59</v>
+      </c>
+      <c r="D18" s="26"/>
+    </row>
+    <row r="19" ht="18" customHeight="1" spans="2:4">
+      <c r="B19" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="C18" s="25" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="19" ht="18" customHeight="1" spans="2:3">
-      <c r="B19" s="24" t="s">
+      <c r="C19" s="25" t="s">
         <v>62</v>
       </c>
-      <c r="C19" s="25" t="s">
+      <c r="D19" s="26"/>
+    </row>
+    <row r="20" ht="18" customHeight="1" spans="2:4">
+      <c r="B20" s="24" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="20" ht="18" customHeight="1" spans="2:3">
-      <c r="B20" s="24" t="s">
+      <c r="C20" s="25" t="s">
+        <v>62</v>
+      </c>
+      <c r="D20" s="26"/>
+    </row>
+    <row r="21" ht="18" customHeight="1" spans="2:4">
+      <c r="B21" s="24" t="s">
+        <v>47</v>
+      </c>
+      <c r="C21" s="25" t="s">
+        <v>49</v>
+      </c>
+      <c r="D21" s="26"/>
+    </row>
+    <row r="22" ht="18" customHeight="1" spans="2:4">
+      <c r="B22" s="24" t="s">
         <v>64</v>
       </c>
-      <c r="C20" s="25" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="21" ht="18" customHeight="1" spans="2:3">
-      <c r="B21" s="24" t="s">
-        <v>48</v>
-      </c>
-      <c r="C21" s="25" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="22" ht="18" customHeight="1" spans="2:3">
-      <c r="B22" s="24" t="s">
-        <v>65</v>
-      </c>
       <c r="C22" s="25" t="s">
-        <v>50</v>
-      </c>
+        <v>49</v>
+      </c>
+      <c r="D22" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -3490,39 +3566,39 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:11">
       <c r="A1" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:11">
       <c r="A2" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="I2" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="J2" s="2" t="s">
         <v>75</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>76</v>
       </c>
       <c r="K2" s="2" t="s">
         <v>18</v>
@@ -3530,315 +3606,315 @@
     </row>
     <row r="3" ht="168" customHeight="1" spans="1:11">
       <c r="A3" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="F3" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="G3" s="3" t="s">
         <v>82</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>83</v>
       </c>
       <c r="H3" s="3"/>
       <c r="I3" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J3" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="K3" s="3" t="s">
         <v>84</v>
-      </c>
-      <c r="K3" s="3" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="4" ht="123" customHeight="1" spans="1:11">
       <c r="A4" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="C4" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="B4" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C4" s="6" t="s">
+      <c r="D4" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="E4" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="F4" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="G4" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="H4" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="J4" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="K4" s="6" t="s">
         <v>91</v>
-      </c>
-      <c r="H4" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="J4" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="K4" s="6" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="5" ht="151" customHeight="1" spans="1:11">
       <c r="A5" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="C5" s="3" t="s">
+      <c r="D5" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="E5" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="F5" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="G5" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="H5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="J5" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="H5" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="J5" s="8" t="s">
+      <c r="K5" s="3" t="s">
         <v>99</v>
-      </c>
-      <c r="K5" s="3" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="6" ht="132" customHeight="1" spans="1:11">
       <c r="A6" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="C6" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="B6" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C6" s="6" t="s">
+      <c r="D6" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="E6" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="D6" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="E6" s="6" t="s">
+      <c r="F6" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="G6" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="H6" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="J6" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="K6" s="6" t="s">
         <v>105</v>
-      </c>
-      <c r="H6" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="I6" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="J6" s="9" t="s">
-        <v>99</v>
-      </c>
-      <c r="K6" s="6" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="7" ht="176" customHeight="1" spans="1:11">
       <c r="A7" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="C7" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="D7" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="E7" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="F7" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="G7" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="G7" s="3" t="s">
+      <c r="H7" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="J7" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="K7" s="3" t="s">
         <v>113</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="I7" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="J7" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="K7" s="3" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="8" ht="151" customHeight="1" spans="1:11">
       <c r="A8" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="C8" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="B8" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="C8" s="6" t="s">
+      <c r="D8" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="E8" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="D8" s="6" t="s">
-        <v>110</v>
-      </c>
-      <c r="E8" s="6" t="s">
+      <c r="F8" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="G8" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="G8" s="6" t="s">
+      <c r="H8" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="J8" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="K8" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="H8" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="I8" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="J8" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="K8" s="6" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="9" ht="146" customHeight="1" spans="1:11">
       <c r="A9" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="C9" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="B9" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="C9" s="3" t="s">
+      <c r="D9" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="E9" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="F9" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="F9" s="3" t="s">
+      <c r="G9" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="G9" s="3" t="s">
-        <v>126</v>
-      </c>
       <c r="H9" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J9" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="10" ht="167" customHeight="1" spans="1:11">
       <c r="A10" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="B10" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="C10" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="D10" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="E10" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="F10" s="6" t="s">
         <v>131</v>
       </c>
-      <c r="F10" s="6" t="s">
+      <c r="G10" s="6" t="s">
         <v>132</v>
       </c>
-      <c r="G10" s="6" t="s">
+      <c r="H10" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="I10" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="J10" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="K10" s="6" t="s">
         <v>133</v>
-      </c>
-      <c r="H10" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="I10" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="J10" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="K10" s="6" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="11" ht="183" customHeight="1" spans="1:11">
       <c r="A11" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="B11" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="C11" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="D11" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="E11" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="F11" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="F11" s="3" t="s">
+      <c r="G11" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="G11" s="3" t="s">
+      <c r="H11" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I11" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="J11" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="K11" s="3" t="s">
         <v>141</v>
-      </c>
-      <c r="H11" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="I11" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="J11" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="K11" s="3" t="s">
-        <v>142</v>
       </c>
     </row>
   </sheetData>
@@ -3852,6 +3928,354 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:K10"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="3" width="32" customWidth="1"/>
+    <col min="4" max="4" width="30" customWidth="1"/>
+    <col min="5" max="5" width="52" customWidth="1"/>
+    <col min="6" max="6" width="38" customWidth="1"/>
+    <col min="7" max="7" width="44" customWidth="1"/>
+    <col min="8" max="8" width="22" customWidth="1"/>
+    <col min="9" max="9" width="13" customWidth="1"/>
+    <col min="10" max="10" width="12" customWidth="1"/>
+    <col min="11" max="11" width="24" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1" spans="1:11">
+      <c r="A1" s="1" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1" spans="1:11">
+      <c r="A2" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" ht="65" customHeight="1" spans="1:11">
+      <c r="A3" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="4" ht="65" customHeight="1" spans="1:11">
+      <c r="A4" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="J4" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="K4" s="6" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="5" ht="65" customHeight="1" spans="1:11">
+      <c r="A5" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="6" ht="65" customHeight="1" spans="1:11">
+      <c r="A6" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="J6" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="K6" s="6" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="7" ht="65" customHeight="1" spans="1:11">
+      <c r="A7" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="J7" s="10" t="s">
+        <v>181</v>
+      </c>
+      <c r="K7" s="3" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="8" ht="65" customHeight="1" spans="1:11">
+      <c r="A8" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>187</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="H8" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="J8" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="K8" s="6" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="9" ht="65" customHeight="1" spans="1:11">
+      <c r="A9" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I9" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="J9" s="10" t="s">
+        <v>181</v>
+      </c>
+      <c r="K9" s="3" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="10" ht="36" spans="1:11">
+      <c r="A10" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I10" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="J10" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="K10" s="3" t="s">
+        <v>202</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:K1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:K9"/>
@@ -3872,39 +4296,39 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:11">
       <c r="A1" s="1" t="s">
-        <v>143</v>
+        <v>203</v>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:11">
       <c r="A2" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="I2" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="J2" s="2" t="s">
         <v>75</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>76</v>
       </c>
       <c r="K2" s="2" t="s">
         <v>18</v>
@@ -3912,525 +4336,247 @@
     </row>
     <row r="3" ht="65" customHeight="1" spans="1:11">
       <c r="A3" s="3" t="s">
-        <v>144</v>
+        <v>204</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>145</v>
+        <v>205</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>146</v>
+        <v>206</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>147</v>
+        <v>207</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>148</v>
+        <v>208</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>149</v>
+        <v>209</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>150</v>
+        <v>210</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>151</v>
+        <v>211</v>
       </c>
     </row>
     <row r="4" ht="65" customHeight="1" spans="1:11">
       <c r="A4" s="6" t="s">
-        <v>152</v>
+        <v>212</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>153</v>
+        <v>213</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>154</v>
+        <v>214</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>155</v>
+        <v>215</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>156</v>
+        <v>216</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>157</v>
+        <v>217</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>158</v>
+        <v>218</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="K4" s="6" t="s">
-        <v>159</v>
+        <v>219</v>
       </c>
     </row>
     <row r="5" ht="65" customHeight="1" spans="1:11">
       <c r="A5" s="3" t="s">
-        <v>160</v>
+        <v>220</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>161</v>
+        <v>221</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>162</v>
+        <v>222</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>163</v>
+        <v>223</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>164</v>
+        <v>224</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>165</v>
+        <v>225</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>166</v>
+        <v>226</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="J5" s="5" t="s">
-        <v>84</v>
+        <v>44</v>
+      </c>
+      <c r="J5" s="8" t="s">
+        <v>98</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>167</v>
+        <v>227</v>
       </c>
     </row>
     <row r="6" ht="65" customHeight="1" spans="1:11">
       <c r="A6" s="6" t="s">
-        <v>168</v>
+        <v>228</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>169</v>
+        <v>229</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>170</v>
+        <v>230</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>171</v>
+        <v>231</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>172</v>
+        <v>232</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>173</v>
+        <v>233</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>174</v>
+        <v>234</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J6" s="9" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="K6" s="6" t="s">
-        <v>175</v>
+        <v>235</v>
       </c>
     </row>
     <row r="7" ht="65" customHeight="1" spans="1:11">
       <c r="A7" s="3" t="s">
-        <v>176</v>
+        <v>236</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>169</v>
+        <v>237</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>177</v>
+        <v>238</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>178</v>
+        <v>239</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>179</v>
+        <v>240</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>180</v>
+        <v>241</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>181</v>
+        <v>242</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="J7" s="10" t="s">
-        <v>182</v>
+        <v>44</v>
+      </c>
+      <c r="J7" s="5" t="s">
+        <v>83</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>183</v>
+        <v>243</v>
       </c>
     </row>
     <row r="8" ht="65" customHeight="1" spans="1:11">
       <c r="A8" s="6" t="s">
-        <v>184</v>
+        <v>244</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>169</v>
+        <v>245</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>185</v>
+        <v>246</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>186</v>
+        <v>247</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>187</v>
+        <v>248</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>188</v>
+        <v>249</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>189</v>
+        <v>250</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="J8" s="7" t="s">
-        <v>84</v>
+        <v>44</v>
+      </c>
+      <c r="J8" s="9" t="s">
+        <v>98</v>
       </c>
       <c r="K8" s="6" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="9" ht="65" customHeight="1" spans="1:11">
-      <c r="A9" s="3" t="s">
-        <v>191</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>169</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>194</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>195</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>196</v>
-      </c>
-      <c r="H9" s="3" t="s">
-        <v>23</v>
+        <v>251</v>
+      </c>
+    </row>
+    <row r="9" ht="24" spans="1:11">
+      <c r="A9" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>252</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>254</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>256</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>257</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="J9" s="10" t="s">
-        <v>182</v>
-      </c>
-      <c r="K9" s="3" t="s">
-        <v>197</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:K1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:K8"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="7"/>
-  <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="22" customWidth="1"/>
-    <col min="3" max="3" width="32" customWidth="1"/>
-    <col min="4" max="4" width="30" customWidth="1"/>
-    <col min="5" max="5" width="52" customWidth="1"/>
-    <col min="6" max="6" width="38" customWidth="1"/>
-    <col min="7" max="7" width="44" customWidth="1"/>
-    <col min="8" max="8" width="22" customWidth="1"/>
-    <col min="9" max="9" width="13" customWidth="1"/>
-    <col min="10" max="10" width="12" customWidth="1"/>
-    <col min="11" max="11" width="24" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="2" ht="30" customHeight="1" spans="1:11">
-      <c r="A2" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="3" ht="65" customHeight="1" spans="1:11">
-      <c r="A3" s="3" t="s">
-        <v>199</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>200</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>203</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>204</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>205</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="I3" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="J3" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="K3" s="3" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="4" ht="65" customHeight="1" spans="1:11">
-      <c r="A4" s="6" t="s">
-        <v>207</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>208</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>209</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>210</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>211</v>
-      </c>
-      <c r="F4" s="6" t="s">
-        <v>212</v>
-      </c>
-      <c r="G4" s="6" t="s">
-        <v>213</v>
-      </c>
-      <c r="H4" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="J4" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="K4" s="6" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="5" ht="65" customHeight="1" spans="1:11">
-      <c r="A5" s="3" t="s">
-        <v>215</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>216</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>217</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>218</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>219</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>221</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="J5" s="8" t="s">
-        <v>99</v>
-      </c>
-      <c r="K5" s="3" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="6" ht="65" customHeight="1" spans="1:11">
-      <c r="A6" s="6" t="s">
-        <v>223</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>224</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>225</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>226</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>227</v>
-      </c>
-      <c r="F6" s="6" t="s">
-        <v>228</v>
-      </c>
-      <c r="G6" s="6" t="s">
-        <v>229</v>
-      </c>
-      <c r="H6" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="I6" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="J6" s="9" t="s">
-        <v>99</v>
-      </c>
-      <c r="K6" s="6" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="7" ht="65" customHeight="1" spans="1:11">
-      <c r="A7" s="3" t="s">
-        <v>231</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>232</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>233</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>234</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>236</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>237</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="I7" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="J7" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="K7" s="3" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="8" ht="65" customHeight="1" spans="1:11">
-      <c r="A8" s="6" t="s">
-        <v>239</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>240</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>241</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>242</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>243</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>244</v>
-      </c>
-      <c r="G8" s="6" t="s">
-        <v>245</v>
-      </c>
-      <c r="H8" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="I8" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="J8" s="9" t="s">
-        <v>99</v>
-      </c>
-      <c r="K8" s="6" t="s">
-        <v>246</v>
+        <v>44</v>
+      </c>
+      <c r="J9" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="K9" s="6" t="s">
+        <v>258</v>
       </c>
     </row>
   </sheetData>
@@ -4463,39 +4609,39 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:11">
       <c r="A1" s="1" t="s">
-        <v>247</v>
+        <v>259</v>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:11">
       <c r="A2" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="I2" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="J2" s="2" t="s">
         <v>75</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>76</v>
       </c>
       <c r="K2" s="2" t="s">
         <v>18</v>
@@ -4503,142 +4649,142 @@
     </row>
     <row r="3" ht="65" customHeight="1" spans="1:11">
       <c r="A3" s="3" t="s">
-        <v>248</v>
+        <v>260</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>249</v>
+        <v>261</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>250</v>
+        <v>262</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>251</v>
+        <v>263</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>252</v>
+        <v>264</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>253</v>
+        <v>265</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>255</v>
+        <v>267</v>
       </c>
     </row>
     <row r="4" ht="65" customHeight="1" spans="1:11">
       <c r="A4" s="6" t="s">
-        <v>256</v>
+        <v>268</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>257</v>
+        <v>269</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>258</v>
+        <v>270</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>259</v>
+        <v>271</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>260</v>
+        <v>272</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>261</v>
+        <v>273</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>262</v>
+        <v>274</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="K4" s="6" t="s">
-        <v>263</v>
+        <v>275</v>
       </c>
     </row>
     <row r="5" ht="65" customHeight="1" spans="1:11">
       <c r="A5" s="3" t="s">
-        <v>264</v>
+        <v>276</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>265</v>
+        <v>277</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>266</v>
+        <v>278</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>267</v>
+        <v>279</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>268</v>
+        <v>280</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>269</v>
+        <v>281</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>270</v>
+        <v>282</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J5" s="8" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>271</v>
+        <v>283</v>
       </c>
     </row>
     <row r="6" ht="65" customHeight="1" spans="1:11">
       <c r="A6" s="6" t="s">
-        <v>272</v>
+        <v>284</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>249</v>
+        <v>261</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>273</v>
+        <v>285</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>274</v>
+        <v>254</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>275</v>
+        <v>286</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>276</v>
+        <v>287</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>277</v>
+        <v>288</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J6" s="9" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="K6" s="6" t="s">
-        <v>278</v>
+        <v>289</v>
       </c>
     </row>
   </sheetData>
@@ -4671,39 +4817,39 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:11">
       <c r="A1" s="1" t="s">
-        <v>279</v>
+        <v>290</v>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:11">
       <c r="A2" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="I2" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="J2" s="2" t="s">
         <v>75</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>76</v>
       </c>
       <c r="K2" s="2" t="s">
         <v>18</v>
@@ -4711,212 +4857,212 @@
     </row>
     <row r="3" ht="65" customHeight="1" spans="1:11">
       <c r="A3" s="3" t="s">
-        <v>280</v>
+        <v>291</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>281</v>
+        <v>292</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>282</v>
+        <v>293</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>274</v>
+        <v>254</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>283</v>
+        <v>294</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>284</v>
+        <v>295</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>285</v>
+        <v>296</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>286</v>
+        <v>297</v>
       </c>
     </row>
     <row r="4" ht="65" customHeight="1" spans="1:11">
       <c r="A4" s="6" t="s">
-        <v>287</v>
+        <v>298</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>288</v>
+        <v>299</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>289</v>
+        <v>300</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>290</v>
+        <v>301</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>291</v>
+        <v>302</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>292</v>
+        <v>303</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>293</v>
+        <v>304</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J4" s="9" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="K4" s="6" t="s">
-        <v>294</v>
+        <v>305</v>
       </c>
     </row>
     <row r="5" ht="65" customHeight="1" spans="1:11">
       <c r="A5" s="3" t="s">
-        <v>295</v>
+        <v>306</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>296</v>
+        <v>307</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>297</v>
+        <v>308</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>298</v>
+        <v>309</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>299</v>
+        <v>310</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>292</v>
+        <v>303</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>300</v>
+        <v>311</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>301</v>
+        <v>312</v>
       </c>
     </row>
     <row r="6" ht="65" customHeight="1" spans="1:11">
       <c r="A6" s="6" t="s">
-        <v>302</v>
+        <v>313</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>303</v>
+        <v>314</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>304</v>
+        <v>315</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>305</v>
+        <v>316</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>306</v>
+        <v>317</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>307</v>
+        <v>318</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>308</v>
+        <v>319</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J6" s="9" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="K6" s="6" t="s">
-        <v>309</v>
+        <v>320</v>
       </c>
     </row>
     <row r="7" ht="65" customHeight="1" spans="1:11">
       <c r="A7" s="3" t="s">
-        <v>310</v>
+        <v>321</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>311</v>
+        <v>322</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>312</v>
+        <v>323</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>313</v>
+        <v>324</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>314</v>
+        <v>325</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>315</v>
+        <v>326</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>316</v>
+        <v>327</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J7" s="8" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>317</v>
+        <v>328</v>
       </c>
     </row>
     <row r="8" ht="65" customHeight="1" spans="1:11">
       <c r="A8" s="6" t="s">
-        <v>318</v>
+        <v>329</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>319</v>
+        <v>330</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>320</v>
+        <v>331</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>321</v>
+        <v>332</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>322</v>
+        <v>333</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>323</v>
+        <v>334</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J8" s="7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="K8" s="6" t="s">
-        <v>324</v>
+        <v>335</v>
       </c>
     </row>
   </sheetData>
@@ -4949,39 +5095,39 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:11">
       <c r="A1" s="1" t="s">
-        <v>325</v>
+        <v>336</v>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:11">
       <c r="A2" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="I2" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="J2" s="2" t="s">
         <v>75</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>76</v>
       </c>
       <c r="K2" s="2" t="s">
         <v>18</v>
@@ -4989,107 +5135,107 @@
     </row>
     <row r="3" ht="65" customHeight="1" spans="1:11">
       <c r="A3" s="3" t="s">
-        <v>326</v>
+        <v>337</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>327</v>
+        <v>338</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>328</v>
+        <v>339</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>329</v>
+        <v>340</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>330</v>
+        <v>341</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>331</v>
+        <v>342</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>332</v>
+        <v>343</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J3" s="8" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>333</v>
+        <v>344</v>
       </c>
     </row>
     <row r="4" ht="65" customHeight="1" spans="1:11">
       <c r="A4" s="6" t="s">
-        <v>334</v>
+        <v>345</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>335</v>
+        <v>346</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>336</v>
+        <v>347</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>274</v>
+        <v>254</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>337</v>
+        <v>348</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>338</v>
+        <v>349</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>339</v>
+        <v>350</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J4" s="9" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="K4" s="6" t="s">
-        <v>340</v>
+        <v>351</v>
       </c>
     </row>
     <row r="5" ht="65" customHeight="1" spans="1:11">
       <c r="A5" s="3" t="s">
-        <v>341</v>
+        <v>352</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>327</v>
+        <v>338</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>342</v>
+        <v>353</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>343</v>
+        <v>354</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>344</v>
+        <v>355</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>345</v>
+        <v>356</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>346</v>
+        <v>357</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J5" s="10" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>347</v>
+        <v>358</v>
       </c>
     </row>
   </sheetData>
@@ -5104,8 +5250,8 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:K7"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="6"/>
+  <dimension ref="A1:K8"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="7"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
@@ -5122,39 +5268,39 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:11">
       <c r="A1" s="1" t="s">
-        <v>348</v>
+        <v>359</v>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:11">
       <c r="A2" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="I2" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="J2" s="2" t="s">
         <v>75</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>76</v>
       </c>
       <c r="K2" s="2" t="s">
         <v>18</v>
@@ -5162,177 +5308,212 @@
     </row>
     <row r="3" ht="65" customHeight="1" spans="1:11">
       <c r="A3" s="3" t="s">
-        <v>349</v>
+        <v>360</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>350</v>
+        <v>361</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>351</v>
+        <v>362</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>352</v>
+        <v>363</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>353</v>
+        <v>364</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>354</v>
+        <v>365</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>355</v>
+        <v>366</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>356</v>
+        <v>367</v>
       </c>
     </row>
     <row r="4" ht="65" customHeight="1" spans="1:11">
       <c r="A4" s="6" t="s">
-        <v>357</v>
+        <v>368</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>350</v>
+        <v>361</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>358</v>
+        <v>369</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>359</v>
+        <v>370</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>360</v>
+        <v>371</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>361</v>
+        <v>372</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>362</v>
+        <v>373</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="K4" s="6" t="s">
-        <v>363</v>
+        <v>374</v>
       </c>
     </row>
     <row r="5" ht="65" customHeight="1" spans="1:11">
       <c r="A5" s="3" t="s">
-        <v>364</v>
+        <v>375</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>365</v>
+        <v>376</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>366</v>
+        <v>377</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>367</v>
+        <v>378</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>368</v>
+        <v>379</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>369</v>
+        <v>380</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>370</v>
+        <v>381</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>371</v>
+        <v>382</v>
       </c>
     </row>
     <row r="6" ht="65" customHeight="1" spans="1:11">
       <c r="A6" s="6" t="s">
-        <v>372</v>
+        <v>383</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>373</v>
+        <v>384</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>374</v>
+        <v>385</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>375</v>
+        <v>386</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>376</v>
+        <v>387</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>377</v>
+        <v>388</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>378</v>
+        <v>389</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J6" s="7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="K6" s="6" t="s">
-        <v>379</v>
+        <v>390</v>
       </c>
     </row>
     <row r="7" ht="65" customHeight="1" spans="1:11">
       <c r="A7" s="3" t="s">
-        <v>380</v>
+        <v>391</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>381</v>
+        <v>392</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>382</v>
+        <v>393</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>383</v>
+        <v>394</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>384</v>
+        <v>395</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>385</v>
+        <v>396</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>386</v>
+        <v>397</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J7" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>387</v>
+        <v>398</v>
+      </c>
+    </row>
+    <row r="8" ht="36" spans="1:11">
+      <c r="A8" s="3" t="s">
+        <v>391</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>399</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>400</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>378</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>401</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>402</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>403</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="J8" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="K8" s="3" t="s">
+        <v>404</v>
       </c>
     </row>
   </sheetData>

</xml_diff>